<commit_message>
Añadir total vendido con estatus DISPERSADO en Top Estatus
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>id</t>
   </si>
@@ -82,6 +82,12 @@
     <t>antiguedad_cuenta</t>
   </si>
   <si>
+    <t>usuario_cipre</t>
+  </si>
+  <si>
+    <t>contrasena</t>
+  </si>
+  <si>
     <t>asesor</t>
   </si>
   <si>
@@ -97,85 +103,43 @@
     <t>observaciones</t>
   </si>
   <si>
-    <t>score</t>
-  </si>
-  <si>
-    <t>analista</t>
-  </si>
-  <si>
-    <t>C9998</t>
-  </si>
-  <si>
-    <t>C9999</t>
-  </si>
-  <si>
-    <t>Nuevo</t>
-  </si>
-  <si>
-    <t>MEJORAVIT</t>
-  </si>
-  <si>
-    <t>LEADS</t>
-  </si>
-  <si>
-    <t>Prueba Uno</t>
-  </si>
-  <si>
-    <t>Prueba Dos</t>
-  </si>
-  <si>
-    <t>555000111</t>
-  </si>
-  <si>
-    <t>555000222</t>
-  </si>
-  <si>
-    <t>BeworkEdoMex</t>
-  </si>
-  <si>
-    <t>1000</t>
-  </si>
-  <si>
-    <t>5000</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>Soltero</t>
-  </si>
-  <si>
-    <t>Propia</t>
-  </si>
-  <si>
-    <t>uno@example.com</t>
-  </si>
-  <si>
-    <t>Ref Uno</t>
-  </si>
-  <si>
-    <t>111111</t>
-  </si>
-  <si>
-    <t>Hijo</t>
-  </si>
-  <si>
-    <t>Ref Dos</t>
-  </si>
-  <si>
-    <t>222222</t>
-  </si>
-  <si>
-    <t>Amig@</t>
-  </si>
-  <si>
-    <t>2 años</t>
-  </si>
-  <si>
-    <t>2025-12-11</t>
-  </si>
-  <si>
-    <t>DISPERSADO</t>
+    <t>fase</t>
+  </si>
+  <si>
+    <t>registro_tipo</t>
+  </si>
+  <si>
+    <t>C1000</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Cliente Integración</t>
+  </si>
+  <si>
+    <t>5551234567</t>
+  </si>
+  <si>
+    <t>TOXQUI</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>integracion@test.com</t>
+  </si>
+  <si>
+    <t>Asesor Test</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
+  </si>
+  <si>
+    <t>PENDIENTE CLIENTE</t>
+  </si>
+  <si>
+    <t>Cliente creado por test de integración</t>
   </si>
 </sst>
 </file>
@@ -533,10 +497,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:29">
+    <row r="1" spans="1:31">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -624,141 +588,46 @@
       <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="2" spans="1:29">
+    <row r="2" spans="1:31">
       <c r="A2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>32</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>33</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>34</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" t="s">
         <v>36</v>
       </c>
-      <c r="H2" t="s">
+      <c r="O2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y2" t="s">
         <v>38</v>
       </c>
-      <c r="I2" t="s">
+      <c r="Z2" t="s">
         <v>39</v>
       </c>
-      <c r="K2" t="s">
+      <c r="AB2" t="s">
         <v>40</v>
       </c>
-      <c r="L2" t="s">
+      <c r="AC2" t="s">
         <v>41</v>
-      </c>
-      <c r="M2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N2" t="s">
-        <v>43</v>
-      </c>
-      <c r="O2" t="s">
-        <v>44</v>
-      </c>
-      <c r="P2" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>46</v>
-      </c>
-      <c r="R2" t="s">
-        <v>47</v>
-      </c>
-      <c r="S2" t="s">
-        <v>48</v>
-      </c>
-      <c r="T2" t="s">
-        <v>49</v>
-      </c>
-      <c r="U2" t="s">
-        <v>50</v>
-      </c>
-      <c r="V2" t="s">
-        <v>51</v>
-      </c>
-      <c r="X2" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29">
-      <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" t="s">
-        <v>40</v>
-      </c>
-      <c r="L3" t="s">
-        <v>41</v>
-      </c>
-      <c r="M3" t="s">
-        <v>42</v>
-      </c>
-      <c r="N3" t="s">
-        <v>43</v>
-      </c>
-      <c r="O3" t="s">
-        <v>44</v>
-      </c>
-      <c r="P3" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R3" t="s">
-        <v>47</v>
-      </c>
-      <c r="S3" t="s">
-        <v>48</v>
-      </c>
-      <c r="T3" t="s">
-        <v>49</v>
-      </c>
-      <c r="U3" t="s">
-        <v>50</v>
-      </c>
-      <c r="V3" t="s">
-        <v>51</v>
-      </c>
-      <c r="X3" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>